<commit_message>
feat: add profession selection and weapon loadouts
</commit_message>
<xml_diff>
--- a/Config/Excel/DT_CharacterAttributes.xlsx
+++ b/Config/Excel/DT_CharacterAttributes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\UnrealDeepRock_Config_Preview\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\letsdeeprock-profession-preview\com-final-serial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27185FA0-B679-4B6C-AD4C-7A8D2F7DE242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EC9F193-5B99-4E97-A43B-2E9FDCD8F2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="68">
   <si>
     <t>#TABLE=DT_CharacterAttributes</t>
   </si>
@@ -205,46 +205,28 @@
     <t>幸运值</t>
   </si>
   <si>
+    <t>VisionHalfAngle</t>
+  </si>
+  <si>
+    <t>VisionRange</t>
+  </si>
+  <si>
+    <t>视野半角(朝向左右各扩展角度)</t>
+  </si>
+  <si>
+    <t>最大视野距离(cm，0表示不限制)</t>
+  </si>
+  <si>
     <t>Engineer</t>
-  </si>
-  <si>
-    <t>平衡型，擅长防御工事</t>
-  </si>
-  <si>
-    <t>Scout</t>
-  </si>
-  <si>
-    <t>高机动，擅长侦察探索</t>
-  </si>
-  <si>
-    <t>Driller</t>
-  </si>
-  <si>
-    <t>近战火力，擅长挖掘开路</t>
-  </si>
-  <si>
-    <t>Gunner</t>
-  </si>
-  <si>
-    <t>重火力输出，擅长压制</t>
-  </si>
-  <si>
-    <t>VisionHalfAngle</t>
-  </si>
-  <si>
-    <t>VisionRange</t>
-  </si>
-  <si>
-    <t>视野半角(朝向左右各扩展角度)</t>
-  </si>
-  <si>
-    <t>最大视野距离(cm，0表示不限制)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Demolitionist</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Ranger</t>
-  </si>
-  <si>
-    <t>游侠样板职业</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -609,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:AD8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.625" style="1" customWidth="1"/>
@@ -806,10 +788,10 @@
         <v>33</v>
       </c>
       <c r="AC3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="AD3" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.2">
@@ -898,18 +880,18 @@
         <v>60</v>
       </c>
       <c r="AC4" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="AD4" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -998,91 +980,91 @@
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6">
+        <v>120</v>
+      </c>
+      <c r="D6">
+        <v>40</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>0.05</v>
+      </c>
+      <c r="I6">
+        <v>1.5</v>
+      </c>
+      <c r="J6">
+        <v>0.1</v>
+      </c>
+      <c r="K6">
+        <v>0.15</v>
+      </c>
+      <c r="L6">
+        <v>0.3</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>0.3</v>
+      </c>
+      <c r="O6">
+        <v>0.9</v>
+      </c>
+      <c r="P6">
+        <v>1.2</v>
+      </c>
+      <c r="Q6">
+        <v>500</v>
+      </c>
+      <c r="R6">
+        <v>0.1</v>
+      </c>
+      <c r="S6">
+        <v>0.2</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0.1</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>120</v>
+      </c>
+      <c r="Y6">
+        <v>4</v>
+      </c>
+      <c r="Z6">
         <v>80</v>
       </c>
-      <c r="D6">
-        <v>30</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
+      <c r="AA6">
         <v>2</v>
       </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0.15</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0.1</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>1.2</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>1.3</v>
-      </c>
-      <c r="P6">
-        <v>2</v>
-      </c>
-      <c r="Q6">
-        <v>800</v>
-      </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-      <c r="X6">
-        <v>80</v>
-      </c>
-      <c r="Y6">
-        <v>8</v>
-      </c>
-      <c r="Z6">
-        <v>120</v>
-      </c>
-      <c r="AA6">
-        <v>5</v>
-      </c>
       <c r="AB6">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AC6">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="AD6">
         <v>0</v>
@@ -1090,279 +1072,100 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C7">
+        <v>80</v>
+      </c>
+      <c r="D7">
+        <v>30</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0.15</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0.1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1.2</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>1.3</v>
+      </c>
+      <c r="P7">
+        <v>2</v>
+      </c>
+      <c r="Q7">
+        <v>800</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>80</v>
+      </c>
+      <c r="Y7">
+        <v>8</v>
+      </c>
+      <c r="Z7">
         <v>120</v>
       </c>
-      <c r="D7">
-        <v>40</v>
-      </c>
-      <c r="E7">
-        <v>4</v>
-      </c>
-      <c r="F7">
-        <v>4</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
-        <v>0.05</v>
-      </c>
-      <c r="I7">
-        <v>1.5</v>
-      </c>
-      <c r="J7">
+      <c r="AA7">
+        <v>5</v>
+      </c>
+      <c r="AB7">
         <v>0.1</v>
       </c>
-      <c r="K7">
-        <v>0.15</v>
-      </c>
-      <c r="L7">
-        <v>0.3</v>
-      </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-      <c r="N7">
-        <v>0.3</v>
-      </c>
-      <c r="O7">
-        <v>0.9</v>
-      </c>
-      <c r="P7">
-        <v>1.2</v>
-      </c>
-      <c r="Q7">
-        <v>500</v>
-      </c>
-      <c r="R7">
-        <v>0.1</v>
-      </c>
-      <c r="S7">
-        <v>0.2</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0.1</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-      <c r="X7">
-        <v>120</v>
-      </c>
-      <c r="Y7">
-        <v>4</v>
-      </c>
-      <c r="Z7">
-        <v>80</v>
-      </c>
-      <c r="AA7">
-        <v>2</v>
-      </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
       <c r="AC7">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="AD7">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8">
-        <v>150</v>
-      </c>
-      <c r="D8">
-        <v>60</v>
-      </c>
-      <c r="E8">
-        <v>3</v>
-      </c>
-      <c r="F8">
-        <v>5</v>
-      </c>
-      <c r="G8">
-        <v>15</v>
-      </c>
-      <c r="H8">
-        <v>0.08</v>
-      </c>
-      <c r="I8">
-        <v>1.8</v>
-      </c>
-      <c r="J8">
-        <v>0.2</v>
-      </c>
-      <c r="K8">
-        <v>0.2</v>
-      </c>
-      <c r="L8">
-        <v>0.5</v>
-      </c>
-      <c r="M8">
-        <v>0.8</v>
-      </c>
-      <c r="N8">
-        <v>0.1</v>
-      </c>
-      <c r="O8">
-        <v>0.8</v>
-      </c>
-      <c r="P8">
-        <v>1</v>
-      </c>
-      <c r="Q8">
-        <v>400</v>
-      </c>
-      <c r="R8">
-        <v>0.15</v>
-      </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
-      <c r="T8">
-        <v>0</v>
-      </c>
-      <c r="U8">
-        <v>0</v>
-      </c>
-      <c r="V8">
-        <v>0.15</v>
-      </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-      <c r="X8">
-        <v>80</v>
-      </c>
-      <c r="Y8">
-        <v>3</v>
-      </c>
-      <c r="Z8">
-        <v>100</v>
-      </c>
-      <c r="AA8">
-        <v>3</v>
-      </c>
-      <c r="AB8">
-        <v>0</v>
-      </c>
-      <c r="AC8">
-        <v>50</v>
-      </c>
-      <c r="AD8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="1">
-        <v>80</v>
-      </c>
-      <c r="D9">
-        <v>30</v>
-      </c>
-      <c r="E9">
-        <v>8</v>
-      </c>
-      <c r="F9">
-        <v>2</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>0.15</v>
-      </c>
-      <c r="I9">
-        <v>2</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>0.1</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9">
-        <v>1.2</v>
-      </c>
-      <c r="N9">
-        <v>0</v>
-      </c>
-      <c r="O9">
-        <v>1.3</v>
-      </c>
-      <c r="P9">
-        <v>2</v>
-      </c>
-      <c r="Q9">
-        <v>800</v>
-      </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-      <c r="T9">
-        <v>0</v>
-      </c>
-      <c r="U9">
-        <v>0</v>
-      </c>
-      <c r="V9">
-        <v>0</v>
-      </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
-      <c r="X9">
-        <v>80</v>
-      </c>
-      <c r="Y9">
-        <v>8</v>
-      </c>
-      <c r="Z9">
-        <v>120</v>
-      </c>
-      <c r="AA9">
-        <v>5</v>
-      </c>
-      <c r="AB9">
-        <v>0.1</v>
-      </c>
-      <c r="AC9">
-        <v>75</v>
-      </c>
-      <c r="AD9">
-        <v>0</v>
-      </c>
+      <c r="A8"/>
+      <c r="B8"/>
+      <c r="C8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>